<commit_message>
chore: add custom-CI test result
</commit_message>
<xml_diff>
--- a/scripts/results/known_growth_phenotypes_w_pred.xlsx
+++ b/scripts/results/known_growth_phenotypes_w_pred.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -25,12 +26,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -62,19 +58,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -89,7 +76,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -968,7 +955,7 @@
           <t>(Kratzl, 2026)</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="n">
         <v>0.5649999999999999</v>
       </c>
@@ -1214,7 +1201,7 @@
           <t>(Kratzl, 2026)</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="n">
         <v>0.6870000000000001</v>
       </c>
@@ -2175,7 +2162,7 @@
           <t>(Koch, 2020)</t>
         </is>
       </c>
-      <c r="F53" s="2" t="n"/>
+      <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="n">
         <v>0</v>
       </c>
@@ -2206,8 +2193,8 @@
           <t>Unsure</t>
         </is>
       </c>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n"/>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr"/>
       <c r="G54" s="3" t="n">
         <v>0.585</v>
       </c>
@@ -2238,8 +2225,8 @@
           <t>Unsure</t>
         </is>
       </c>
-      <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="n"/>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr"/>
       <c r="G55" s="3" t="n">
         <v>0</v>
       </c>
@@ -2270,8 +2257,8 @@
           <t>Unsure</t>
         </is>
       </c>
-      <c r="E56" s="3" t="n"/>
-      <c r="F56" s="3" t="n"/>
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="3" t="inlineStr"/>
       <c r="G56" s="3" t="n">
         <v>0.638</v>
       </c>
@@ -2287,7 +2274,7 @@
           <t>Marine Broth (No Nitrogen)</t>
         </is>
       </c>
-      <c r="B57" s="3" t="n"/>
+      <c r="B57" s="3" t="inlineStr"/>
       <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Ammonium, Glucose</t>
@@ -2323,7 +2310,7 @@
           <t>Marine Broth (No Nitrogen)</t>
         </is>
       </c>
-      <c r="B58" s="3" t="n"/>
+      <c r="B58" s="3" t="inlineStr"/>
       <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Ammonium, Pyruvate</t>
@@ -2359,7 +2346,7 @@
           <t>Marine Broth (No Nitrogen)</t>
         </is>
       </c>
-      <c r="B59" s="3" t="n"/>
+      <c r="B59" s="3" t="inlineStr"/>
       <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Nitrate, Glucose</t>
@@ -2395,7 +2382,7 @@
           <t>Marine Broth (No Nitrogen)</t>
         </is>
       </c>
-      <c r="B60" s="3" t="n"/>
+      <c r="B60" s="3" t="inlineStr"/>
       <c r="C60" s="3" t="inlineStr">
         <is>
           <t>Nitrate, Pyruvate</t>
@@ -2431,7 +2418,7 @@
           <t>Marine Broth (No Nitrogen)</t>
         </is>
       </c>
-      <c r="B61" s="3" t="n"/>
+      <c r="B61" s="3" t="inlineStr"/>
       <c r="C61" s="3" t="inlineStr">
         <is>
           <t>Urea+Pyruvate</t>
@@ -2467,7 +2454,7 @@
           <t>Marine Broth (No Nitrogen)</t>
         </is>
       </c>
-      <c r="B62" s="3" t="n"/>
+      <c r="B62" s="3" t="inlineStr"/>
       <c r="C62" s="3" t="inlineStr">
         <is>
           <t>Urea, Glucose</t>
@@ -2498,6 +2485,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>